<commit_message>
Extend Table F1 to nine item pairs with options and percent correct
Table F1 now shows one bank and one AI-generated item for each demand
level in each test form, with the response options transcribed from the
test instrument and the percentage of students who answered each item
correctly.
</commit_message>
<xml_diff>
--- a/notebook/outputs/tables/paper_tables.xlsx
+++ b/notebook/outputs/tables/paper_tables.xlsx
@@ -1451,218 +1451,791 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Demand</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Keyed answer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Correct responses (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Stem</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Options</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Bank</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Addition and subtraction operations</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="n">
+        <v>92</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Solve 65217 + 26123</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>a) 39094 | b) 91340* | c) 81330 | d) 91330</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>AI-generated</t>
         </is>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Addition and subtraction operations</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="n">
+        <v>90</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>Solve 45 + 27</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>a) 72* | b) 62 | c) 78 | d) 53</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Bank</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>13</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Multiplicative problems</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="n">
+        <v>38</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>There are 30 students in a class. The ratio of boys to girls in the class is 2 to 3. How many boys are in the class?</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>a) 6 | b) 12* | c) 18 | d) 20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>AI-generated</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>14</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Multiplicative problems</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="n">
+        <v>58</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>A bicycle costs 120 dollars and there is a 25% discount. What is the discounted price?</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>a) 105 | b) 90* | c) 120 | d) 150</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Bank</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>21</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Multiplicative problems</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="n">
+        <v>33</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>A represents the number of magazines Lina reads each week. Which of these expressions represents the total number of magazines she reads in 6 weeks?</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>a) 6 + A | b) 6 × A* | c) A + 6 | d) (A + A) × 6</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>AI-generated</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="D7" t="n">
         <v>22</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Multiplicative problems</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="n">
+        <v>19</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>In a basket there are apples and oranges in the ratio 3:5. If there are 64 pieces in total, how many are oranges?</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>a) 24 | b) 40* | c) 32 | d) 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Addition and subtraction operations</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>84</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Solve 72 - 25</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>a) 47* | b) 57 | c) 87 | d) 97</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AI-generated</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Addition and subtraction operations</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>86</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Solve 126 - 58</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>a) 58 | b) 68* | c) 76 | d) 66</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>52</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>In a garden there are 14 columns of plants and each column has 20 plants. Then, a gardener plants 6 more columns and each column has 20 plants. How many plants are there in total in the garden now?</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>a) 280 | b) 300 | c) 400* | d) 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AI-generated</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>62</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>In a bag there are 48 candies. If they are shared among 6 children, how many candies does each one receive?</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>a) 6 | b) 7 | c) 8* | d) 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>23</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>71</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>It takes Chris 4 minutes to wash one window. He wants to know how many minutes it will take him to wash 8 windows at that same rate. He should:</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>a) multiply 4 × 8* | b) divide 8 by 4 | c) subtract 4 from 8 | d) add 8 and 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>AI-generated</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>22</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>26</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>A fair gives away balloons in the ratio 4:1:2 for the colors red, green, and blue. If 70 balloons are given away in total, how many are green?</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>a) 10* | b) 40 | c) 14 | d) 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Addition and subtraction operations</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>63</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Solve: 65827 + 63503 - 100298</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>a) 29032* | b) 29168 | c) 102623 | d) 129330</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>AI-generated</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Addition and subtraction operations</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>81</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Solve 87 - 29</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>a) 58* | b) 57 | c) 68 | d) 97</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>13</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>25</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>An alloy is made of gold and silver in the ratio of 1 gram of gold per 4 grams of silver. What is the weight, in grams, of the silver in 40 grams of this alloy?</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>a) 8 | b) 32* | c) 10 | d) 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AI-generated</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>12</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>76</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>In a library there are 7 shelves and each shelf has 8 books. How many books are there in total?</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>a) 54 | b) 56* | c) 64 | d) 48</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>25</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>c</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>46</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Mark's garden has 84 rows of cabbages. There are 57 cabbages in each row. What is the best way to estimate the total?</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>a) 100 × 50 = 5000 | b) 90 × 60 = 5400 | c) 80 × 60 = 4800* | d) 80 × 50 = 4000</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AI-generated</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>26</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Multiplicative problems</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>40</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>On a shelf, the colors of the trays repeat in the order red, green, blue. If the trays are numbered starting from 1, what color is tray number 53?</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>a) red | b) green* | c) blue | d) yellow</t>
         </is>
       </c>
     </row>

</xml_diff>